<commit_message>
Corrida | SFE-PATM | 2026-06-17 12:05:59.277667
</commit_message>
<xml_diff>
--- a/indicadores/SFE-PATM_out.xlsx
+++ b/indicadores/SFE-PATM_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="310">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Patentamiento de maquinaria en Santa Fe</t>
+    <t xml:space="preserve">Patentamiento de maquinaria</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">const | td1coef</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">08/06/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">arodriguez</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1440,9 +1446,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1453,7 +1463,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1467,7 +1477,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
@@ -1483,7 +1493,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1511,7 +1521,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1525,7 +1535,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
@@ -1553,7 +1563,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -1567,7 +1577,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -1581,7 +1591,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -1595,7 +1605,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -1611,7 +1621,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -1625,7 +1635,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -1773,10 +1783,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -1789,10 +1799,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -1816,66 +1826,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>107</v>
@@ -1928,7 +1938,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>97</v>
@@ -1985,7 +1995,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>99</v>
@@ -2042,7 +2052,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>144</v>
@@ -2099,7 +2109,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>189</v>
@@ -2156,7 +2166,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>154</v>
@@ -2213,7 +2223,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>189</v>
@@ -2270,7 +2280,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>206</v>
@@ -2327,7 +2337,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>189</v>
@@ -2384,7 +2394,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>226</v>
@@ -2441,7 +2451,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>154</v>
@@ -2498,7 +2508,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>166</v>
@@ -2555,7 +2565,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>118</v>
@@ -2614,7 +2624,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>126</v>
@@ -2673,7 +2683,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>84</v>
@@ -2732,7 +2742,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>111</v>
@@ -2791,7 +2801,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>123</v>
@@ -2850,7 +2860,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>109</v>
@@ -2909,7 +2919,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>123</v>
@@ -2968,7 +2978,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>121</v>
@@ -3027,7 +3037,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>148</v>
@@ -3086,7 +3096,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>144</v>
@@ -3145,7 +3155,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>106</v>
@@ -3204,7 +3214,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>131</v>
@@ -3263,7 +3273,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>104</v>
@@ -3322,7 +3332,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>76</v>
@@ -3381,7 +3391,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>103</v>
@@ -3440,7 +3450,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>129</v>
@@ -3499,7 +3509,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>101</v>
@@ -3558,7 +3568,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>133</v>
@@ -3617,7 +3627,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>107</v>
@@ -3676,7 +3686,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>70</v>
@@ -3735,7 +3745,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>104</v>
@@ -3794,7 +3804,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>140</v>
@@ -3853,7 +3863,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>133</v>
@@ -3912,7 +3922,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>132</v>
@@ -3971,7 +3981,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>68</v>
@@ -4030,7 +4040,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>82</v>
@@ -4089,7 +4099,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>74</v>
@@ -4148,7 +4158,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>112</v>
@@ -4207,7 +4217,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>122</v>
@@ -4266,7 +4276,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>114</v>
@@ -4325,7 +4335,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>91</v>
@@ -4384,7 +4394,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>138</v>
@@ -4443,7 +4453,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>131</v>
@@ -4502,7 +4512,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>171</v>
@@ -4561,7 +4571,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>160</v>
@@ -4620,7 +4630,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>198</v>
@@ -4679,7 +4689,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>163</v>
@@ -4738,7 +4748,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>94</v>
@@ -4797,7 +4807,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>148</v>
@@ -4856,7 +4866,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>134</v>
@@ -4915,7 +4925,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>159</v>
@@ -4974,7 +4984,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>192</v>
@@ -5033,7 +5043,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>145</v>
@@ -5092,7 +5102,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>177</v>
@@ -5151,7 +5161,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>175</v>
@@ -5210,7 +5220,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>192</v>
@@ -5269,7 +5279,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>214</v>
@@ -5328,7 +5338,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>217</v>
@@ -5387,7 +5397,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>151</v>
@@ -5446,7 +5456,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>100</v>
@@ -5505,7 +5515,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>139</v>
@@ -5564,7 +5574,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>129</v>
@@ -5623,7 +5633,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>162</v>
@@ -5682,7 +5692,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>122</v>
@@ -5741,7 +5751,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>121</v>
@@ -5800,7 +5810,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>138</v>
@@ -5859,7 +5869,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>117</v>
@@ -5918,7 +5928,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>144</v>
@@ -5977,7 +5987,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>108</v>
@@ -6036,7 +6046,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>130</v>
@@ -6095,7 +6105,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>88</v>
@@ -6154,7 +6164,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>90</v>
@@ -6213,7 +6223,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>92</v>
@@ -6272,7 +6282,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>91</v>
@@ -6331,7 +6341,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>115</v>
@@ -6390,7 +6400,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>107</v>
@@ -6449,7 +6459,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>111</v>
@@ -6508,7 +6518,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>133</v>
@@ -6567,7 +6577,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>145</v>
@@ -6626,7 +6636,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>144</v>
@@ -6685,7 +6695,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>109</v>
@@ -6744,7 +6754,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>107</v>
@@ -6803,7 +6813,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>124</v>
@@ -6862,7 +6872,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>81</v>
@@ -6921,7 +6931,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>63</v>
@@ -6980,7 +6990,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>20</v>
@@ -7039,7 +7049,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>113</v>
@@ -7098,7 +7108,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>126</v>
@@ -7157,7 +7167,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>173</v>
@@ -7216,7 +7226,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>151</v>
@@ -7275,7 +7285,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>161</v>
@@ -7334,7 +7344,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>149</v>
@@ -7393,7 +7403,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>156</v>
@@ -7452,7 +7462,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>167</v>
@@ -7511,7 +7521,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>106</v>
@@ -7570,7 +7580,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>120</v>
@@ -7629,7 +7639,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>183</v>
@@ -7688,7 +7698,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>119</v>
@@ -7747,7 +7757,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>115</v>
@@ -7806,7 +7816,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>154</v>
@@ -7865,7 +7875,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>187</v>
@@ -7924,7 +7934,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>187</v>
@@ -7983,7 +7993,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>187</v>
@@ -8042,7 +8052,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>228</v>
@@ -8101,7 +8111,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>230</v>
@@ -8160,7 +8170,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>179</v>
@@ -8219,7 +8229,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>146</v>
@@ -8278,7 +8288,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>128</v>
@@ -8337,7 +8347,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>122</v>
@@ -8396,7 +8406,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>192</v>
@@ -8455,7 +8465,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>224</v>
@@ -8514,7 +8524,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>184</v>
@@ -8573,7 +8583,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>224</v>
@@ -8632,7 +8642,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>229</v>
@@ -8691,7 +8701,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>194</v>
@@ -8750,7 +8760,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>158</v>
@@ -8809,7 +8819,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>153</v>
@@ -8868,7 +8878,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>146</v>
@@ -8927,7 +8937,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>137</v>
@@ -8986,7 +8996,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>112</v>
@@ -9045,7 +9055,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>157</v>
@@ -9104,7 +9114,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>156</v>
@@ -9163,7 +9173,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>160</v>
@@ -9222,7 +9232,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>120</v>
@@ -9281,7 +9291,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>153</v>
@@ -9340,7 +9350,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>153</v>
@@ -9399,7 +9409,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>137</v>
@@ -9458,7 +9468,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>138</v>
@@ -9517,7 +9527,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>136</v>
@@ -9576,7 +9586,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>117</v>
@@ -9635,7 +9645,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>88</v>
@@ -9694,7 +9704,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>74</v>
@@ -9753,7 +9763,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>71</v>
@@ -9812,7 +9822,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>106</v>
@@ -9871,7 +9881,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>137</v>
@@ -9930,7 +9940,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>81</v>
@@ -9989,7 +9999,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>160</v>
@@ -10048,7 +10058,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>250</v>
@@ -10107,7 +10117,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>173</v>
@@ -10166,7 +10176,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>188</v>
@@ -10225,7 +10235,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>178</v>
@@ -10284,7 +10294,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>170</v>
@@ -10343,7 +10353,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>190</v>
@@ -10402,7 +10412,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>160</v>
@@ -10461,7 +10471,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>145</v>
@@ -10520,7 +10530,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>236</v>
@@ -10579,7 +10589,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>276</v>
@@ -10638,7 +10648,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>201</v>
@@ -10697,7 +10707,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>228</v>
@@ -10756,7 +10766,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>224</v>
@@ -10815,7 +10825,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>247</v>
@@ -10874,7 +10884,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>225</v>
@@ -10933,7 +10943,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>190</v>
@@ -10992,7 +11002,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>150</v>
@@ -11051,7 +11061,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>169</v>
@@ -11110,7 +11120,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>145</v>
@@ -11169,7 +11179,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>164</v>
@@ -11228,7 +11238,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>261</v>
@@ -11287,7 +11297,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>269</v>
@@ -11346,7 +11356,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2"/>
       <c r="C163" s="3" t="n">
@@ -11379,7 +11389,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2"/>
       <c r="C164" s="3" t="n">
@@ -11412,7 +11422,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2"/>
       <c r="C165" s="3" t="n">
@@ -11445,7 +11455,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2"/>
       <c r="C166" s="3" t="n">
@@ -11478,7 +11488,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2"/>
       <c r="C167" s="3" t="n">
@@ -11511,7 +11521,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2"/>
       <c r="C168" s="3" t="n">
@@ -11544,7 +11554,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2"/>
       <c r="C169" s="3" t="n">
@@ -11577,7 +11587,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2"/>
       <c r="C170" s="3" t="n">
@@ -11610,7 +11620,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2"/>
       <c r="C171" s="3" t="n">
@@ -11643,7 +11653,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2"/>
       <c r="C172" s="3" t="n">
@@ -11676,7 +11686,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2"/>
       <c r="C173" s="3" t="n">
@@ -11709,7 +11719,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2"/>
       <c r="C174" s="3" t="n">
@@ -11742,7 +11752,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2"/>
       <c r="C175" s="3"/>
@@ -11765,7 +11775,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2"/>
       <c r="C176" s="3"/>
@@ -11788,7 +11798,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2"/>
       <c r="C177" s="3"/>
@@ -11811,7 +11821,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2"/>
       <c r="C178" s="3"/>
@@ -11834,7 +11844,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2"/>
       <c r="C179" s="3"/>
@@ -11857,7 +11867,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2"/>
       <c r="C180" s="3"/>
@@ -11880,7 +11890,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2"/>
       <c r="C181" s="3"/>
@@ -11903,7 +11913,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2"/>
       <c r="C182" s="3"/>
@@ -11926,7 +11936,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2"/>
       <c r="C183" s="3"/>
@@ -11949,7 +11959,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2"/>
       <c r="C184" s="3"/>
@@ -11972,7 +11982,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2"/>
       <c r="C185" s="3"/>
@@ -11995,7 +12005,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2"/>
       <c r="C186" s="3"/>
@@ -12018,7 +12028,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2"/>
       <c r="C187" s="3"/>
@@ -12041,7 +12051,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2"/>
       <c r="C188" s="3"/>
@@ -12064,7 +12074,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2"/>
       <c r="C189" s="3"/>
@@ -12087,7 +12097,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2"/>
       <c r="C190" s="3"/>
@@ -12110,7 +12120,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2"/>
       <c r="C191" s="3"/>
@@ -12133,7 +12143,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2"/>
       <c r="C192" s="3"/>
@@ -12156,7 +12166,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2"/>
       <c r="C193" s="3"/>
@@ -12179,7 +12189,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2"/>
       <c r="C194" s="3"/>
@@ -12202,7 +12212,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2"/>
       <c r="C195" s="3"/>
@@ -12225,7 +12235,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2"/>
       <c r="C196" s="3"/>
@@ -12248,7 +12258,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2"/>
       <c r="C197" s="3"/>
@@ -12271,7 +12281,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2"/>
       <c r="C198" s="3"/>
@@ -12294,7 +12304,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2"/>
       <c r="C199" s="3"/>
@@ -12317,7 +12327,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2"/>
       <c r="C200" s="3"/>
@@ -12340,7 +12350,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2"/>
       <c r="C201" s="3"/>
@@ -12363,7 +12373,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2"/>
       <c r="C202" s="3"/>
@@ -12386,7 +12396,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2"/>
       <c r="C203" s="3"/>
@@ -12409,7 +12419,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2"/>
       <c r="C204" s="3"/>
@@ -12432,7 +12442,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2"/>
       <c r="C205" s="3"/>
@@ -12455,7 +12465,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2"/>
       <c r="C206" s="3"/>
@@ -12478,7 +12488,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2"/>
       <c r="C207" s="3"/>
@@ -12501,7 +12511,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2"/>
       <c r="C208" s="3"/>
@@ -12524,7 +12534,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2"/>
       <c r="C209" s="3"/>
@@ -12547,7 +12557,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2"/>
       <c r="C210" s="3"/>
@@ -12570,7 +12580,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2"/>
       <c r="C211" s="3"/>
@@ -12593,7 +12603,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2"/>
       <c r="C212" s="3"/>
@@ -12616,7 +12626,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2"/>
       <c r="C213" s="3"/>
@@ -12639,7 +12649,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2"/>
       <c r="C214" s="3"/>
@@ -12662,7 +12672,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2"/>
       <c r="C215" s="3"/>
@@ -12685,7 +12695,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2"/>
       <c r="C216" s="3"/>
@@ -12708,7 +12718,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2"/>
       <c r="C217" s="3"/>
@@ -12742,97 +12752,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
   </sheetData>
@@ -12856,7 +12866,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -12866,13 +12876,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>-0.0679309571968585</v>
@@ -12880,7 +12890,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>-0.0322899377937667</v>
@@ -12888,7 +12898,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.0528310048646997</v>
@@ -12896,7 +12906,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.180303130825553</v>
@@ -12904,7 +12914,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.278590409412305</v>
@@ -12912,7 +12922,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.364728068894751</v>
@@ -12920,7 +12930,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.376557100484772</v>
@@ -12928,7 +12938,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.312434802781709</v>
@@ -12936,7 +12946,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.346207131280159</v>
@@ -12944,7 +12954,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.404805158989878</v>
@@ -12952,7 +12962,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.344127890313494</v>
@@ -12960,7 +12970,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.277254569335091</v>
@@ -12968,7 +12978,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.216361346652934</v>
@@ -12976,7 +12986,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0.0885127222757193</v>
@@ -12984,7 +12994,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>-0.0660858204248252</v>
@@ -12992,7 +13002,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>-0.156941271544338</v>
@@ -13000,7 +13010,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>-0.174525208209563</v>
@@ -13008,7 +13018,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>-0.194988574518518</v>
@@ -13016,7 +13026,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>-0.256515493374365</v>
@@ -13047,237 +13057,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6088E16-70EE-4BED-AFF1-9256F331CF5C}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6953032-61F5-49C6-A586-572D4B04EC34}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{999F110C-3575-466E-89F3-40E18EC0A9CE}"/>
 </file>
</xml_diff>